<commit_message>
Ronda 6b: videos de YouTube vinculados a 426 fichas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descargas/catalogo-imex-vigente.xlsx
+++ b/descargas/catalogo-imex-vigente.xlsx
@@ -547,7 +547,11 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1NKruzTqpuM</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -581,7 +585,11 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1NKruzTqpuM</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -615,7 +623,11 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1NKruzTqpuM</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1431,7 +1443,11 @@
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KHXlrnntv7c</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1635,7 +1651,11 @@
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pqiZvjZNDek</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2145,7 +2165,11 @@
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0lK08eUiPwI</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2893,7 +2917,11 @@
         </is>
       </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2927,7 +2955,11 @@
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2961,7 +2993,11 @@
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3029,7 +3065,11 @@
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3063,7 +3103,11 @@
         </is>
       </c>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3097,7 +3141,11 @@
         </is>
       </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3131,7 +3179,11 @@
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3165,7 +3217,11 @@
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3199,7 +3255,11 @@
         </is>
       </c>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3233,7 +3293,11 @@
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3267,7 +3331,11 @@
         </is>
       </c>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3301,7 +3369,11 @@
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3369,7 +3441,11 @@
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3403,7 +3479,11 @@
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3437,7 +3517,11 @@
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3471,7 +3555,11 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3539,7 +3627,11 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3573,7 +3665,11 @@
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3607,7 +3703,11 @@
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3641,7 +3741,11 @@
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3675,7 +3779,11 @@
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3811,7 +3919,11 @@
         </is>
       </c>
       <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3845,7 +3957,11 @@
         </is>
       </c>
       <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3879,7 +3995,11 @@
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3913,7 +4033,11 @@
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4049,7 +4173,11 @@
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4083,7 +4211,11 @@
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4117,7 +4249,11 @@
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4253,7 +4389,11 @@
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w1yNVc_FB2Q</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4831,7 +4971,11 @@
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hz9-cFtvFIw</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5341,7 +5485,11 @@
         </is>
       </c>
       <c r="G144" t="inlineStr"/>
-      <c r="H144" t="inlineStr"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JFQXVx-4N88</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5375,7 +5523,11 @@
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
-      <c r="H145" t="inlineStr"/>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JFQXVx-4N88</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6089,7 +6241,11 @@
         </is>
       </c>
       <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=UVVcpOcyMdM</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7143,7 +7299,11 @@
         </is>
       </c>
       <c r="G197" t="inlineStr"/>
-      <c r="H197" t="inlineStr"/>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WW7U_cQl59A</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -7177,7 +7337,11 @@
         </is>
       </c>
       <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr"/>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Jl7LAjsAUiE</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -7721,7 +7885,11 @@
         </is>
       </c>
       <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr"/>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -8503,7 +8671,11 @@
         </is>
       </c>
       <c r="G237" t="inlineStr"/>
-      <c r="H237" t="inlineStr"/>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=E_Wo40VNrN8</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -8707,7 +8879,11 @@
         </is>
       </c>
       <c r="G243" t="inlineStr"/>
-      <c r="H243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yIw6aSP5730</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -8741,7 +8917,11 @@
         </is>
       </c>
       <c r="G244" t="inlineStr"/>
-      <c r="H244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yIw6aSP5730</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -8775,7 +8955,11 @@
         </is>
       </c>
       <c r="G245" t="inlineStr"/>
-      <c r="H245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yIw6aSP5730</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -9217,7 +9401,11 @@
         </is>
       </c>
       <c r="G258" t="inlineStr"/>
-      <c r="H258" t="inlineStr"/>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -9251,7 +9439,11 @@
         </is>
       </c>
       <c r="G259" t="inlineStr"/>
-      <c r="H259" t="inlineStr"/>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -9285,7 +9477,11 @@
         </is>
       </c>
       <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -9319,7 +9515,11 @@
         </is>
       </c>
       <c r="G261" t="inlineStr"/>
-      <c r="H261" t="inlineStr"/>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -9353,7 +9553,11 @@
         </is>
       </c>
       <c r="G262" t="inlineStr"/>
-      <c r="H262" t="inlineStr"/>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -9387,7 +9591,11 @@
         </is>
       </c>
       <c r="G263" t="inlineStr"/>
-      <c r="H263" t="inlineStr"/>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -10373,7 +10581,11 @@
         </is>
       </c>
       <c r="G292" t="inlineStr"/>
-      <c r="H292" t="inlineStr"/>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rF3yKJPE-c0</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -10611,7 +10823,11 @@
         </is>
       </c>
       <c r="G299" t="inlineStr"/>
-      <c r="H299" t="inlineStr"/>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yDWX4wz9pzQ</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -10645,7 +10861,11 @@
         </is>
       </c>
       <c r="G300" t="inlineStr"/>
-      <c r="H300" t="inlineStr"/>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bbQM8EAEhW4</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -10917,7 +11137,11 @@
         </is>
       </c>
       <c r="G308" t="inlineStr"/>
-      <c r="H308" t="inlineStr"/>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -10951,7 +11175,11 @@
         </is>
       </c>
       <c r="G309" t="inlineStr"/>
-      <c r="H309" t="inlineStr"/>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -10985,7 +11213,11 @@
         </is>
       </c>
       <c r="G310" t="inlineStr"/>
-      <c r="H310" t="inlineStr"/>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -11019,7 +11251,11 @@
         </is>
       </c>
       <c r="G311" t="inlineStr"/>
-      <c r="H311" t="inlineStr"/>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -11053,7 +11289,11 @@
         </is>
       </c>
       <c r="G312" t="inlineStr"/>
-      <c r="H312" t="inlineStr"/>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -11087,7 +11327,11 @@
         </is>
       </c>
       <c r="G313" t="inlineStr"/>
-      <c r="H313" t="inlineStr"/>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -11121,7 +11365,11 @@
         </is>
       </c>
       <c r="G314" t="inlineStr"/>
-      <c r="H314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -11223,7 +11471,11 @@
         </is>
       </c>
       <c r="G317" t="inlineStr"/>
-      <c r="H317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -11257,7 +11509,11 @@
         </is>
       </c>
       <c r="G318" t="inlineStr"/>
-      <c r="H318" t="inlineStr"/>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -11291,7 +11547,11 @@
         </is>
       </c>
       <c r="G319" t="inlineStr"/>
-      <c r="H319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -11325,7 +11585,11 @@
         </is>
       </c>
       <c r="G320" t="inlineStr"/>
-      <c r="H320" t="inlineStr"/>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOt0BPdasdE</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -11733,7 +11997,11 @@
         </is>
       </c>
       <c r="G332" t="inlineStr"/>
-      <c r="H332" t="inlineStr"/>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GX7JX0ApuHk</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -11937,7 +12205,11 @@
         </is>
       </c>
       <c r="G338" t="inlineStr"/>
-      <c r="H338" t="inlineStr"/>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zmozwG1cAGM</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -12345,7 +12617,11 @@
         </is>
       </c>
       <c r="G350" t="inlineStr"/>
-      <c r="H350" t="inlineStr"/>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -12379,7 +12655,11 @@
         </is>
       </c>
       <c r="G351" t="inlineStr"/>
-      <c r="H351" t="inlineStr"/>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -12413,7 +12693,11 @@
         </is>
       </c>
       <c r="G352" t="inlineStr"/>
-      <c r="H352" t="inlineStr"/>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -12447,7 +12731,11 @@
         </is>
       </c>
       <c r="G353" t="inlineStr"/>
-      <c r="H353" t="inlineStr"/>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -12481,7 +12769,11 @@
         </is>
       </c>
       <c r="G354" t="inlineStr"/>
-      <c r="H354" t="inlineStr"/>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -12515,7 +12807,11 @@
         </is>
       </c>
       <c r="G355" t="inlineStr"/>
-      <c r="H355" t="inlineStr"/>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDdof9rPQAw</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -19519,7 +19815,11 @@
         </is>
       </c>
       <c r="G561" t="inlineStr"/>
-      <c r="H561" t="inlineStr"/>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4FEHDl1qdKk</t>
+        </is>
+      </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -19655,7 +19955,11 @@
         </is>
       </c>
       <c r="G565" t="inlineStr"/>
-      <c r="H565" t="inlineStr"/>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rM7Ex77uKSc</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" t="inlineStr">
@@ -19893,7 +20197,11 @@
         </is>
       </c>
       <c r="G572" t="inlineStr"/>
-      <c r="H572" t="inlineStr"/>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
@@ -19927,7 +20235,11 @@
         </is>
       </c>
       <c r="G573" t="inlineStr"/>
-      <c r="H573" t="inlineStr"/>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iN2xYjqUNWI</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -20063,7 +20375,11 @@
         </is>
       </c>
       <c r="G577" t="inlineStr"/>
-      <c r="H577" t="inlineStr"/>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
@@ -20165,7 +20481,11 @@
         </is>
       </c>
       <c r="G580" t="inlineStr"/>
-      <c r="H580" t="inlineStr"/>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OaHOaYSnDfs</t>
+        </is>
+      </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
@@ -20199,7 +20519,11 @@
         </is>
       </c>
       <c r="G581" t="inlineStr"/>
-      <c r="H581" t="inlineStr"/>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
@@ -20535,7 +20859,11 @@
         </is>
       </c>
       <c r="G591" t="inlineStr"/>
-      <c r="H591" t="inlineStr"/>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FjPYNyzWIHE</t>
+        </is>
+      </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -20977,7 +21305,11 @@
         </is>
       </c>
       <c r="G604" t="inlineStr"/>
-      <c r="H604" t="inlineStr"/>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -21011,7 +21343,11 @@
         </is>
       </c>
       <c r="G605" t="inlineStr"/>
-      <c r="H605" t="inlineStr"/>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -21079,7 +21415,11 @@
         </is>
       </c>
       <c r="G607" t="inlineStr"/>
-      <c r="H607" t="inlineStr"/>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
@@ -21113,7 +21453,11 @@
         </is>
       </c>
       <c r="G608" t="inlineStr"/>
-      <c r="H608" t="inlineStr"/>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JWbczacWLGg</t>
+        </is>
+      </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
@@ -21147,7 +21491,11 @@
         </is>
       </c>
       <c r="G609" t="inlineStr"/>
-      <c r="H609" t="inlineStr"/>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -21181,7 +21529,11 @@
         </is>
       </c>
       <c r="G610" t="inlineStr"/>
-      <c r="H610" t="inlineStr"/>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
@@ -21215,7 +21567,11 @@
         </is>
       </c>
       <c r="G611" t="inlineStr"/>
-      <c r="H611" t="inlineStr"/>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -21249,7 +21605,11 @@
         </is>
       </c>
       <c r="G612" t="inlineStr"/>
-      <c r="H612" t="inlineStr"/>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
@@ -21283,7 +21643,11 @@
         </is>
       </c>
       <c r="G613" t="inlineStr"/>
-      <c r="H613" t="inlineStr"/>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
@@ -21317,7 +21681,11 @@
         </is>
       </c>
       <c r="G614" t="inlineStr"/>
-      <c r="H614" t="inlineStr"/>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
@@ -21351,7 +21719,11 @@
         </is>
       </c>
       <c r="G615" t="inlineStr"/>
-      <c r="H615" t="inlineStr"/>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
@@ -21385,7 +21757,11 @@
         </is>
       </c>
       <c r="G616" t="inlineStr"/>
-      <c r="H616" t="inlineStr"/>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
@@ -21419,7 +21795,11 @@
         </is>
       </c>
       <c r="G617" t="inlineStr"/>
-      <c r="H617" t="inlineStr"/>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="618">
       <c r="A618" t="inlineStr">
@@ -21453,7 +21833,11 @@
         </is>
       </c>
       <c r="G618" t="inlineStr"/>
-      <c r="H618" t="inlineStr"/>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
@@ -21487,7 +21871,11 @@
         </is>
       </c>
       <c r="G619" t="inlineStr"/>
-      <c r="H619" t="inlineStr"/>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -21521,7 +21909,11 @@
         </is>
       </c>
       <c r="G620" t="inlineStr"/>
-      <c r="H620" t="inlineStr"/>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -21657,7 +22049,11 @@
         </is>
       </c>
       <c r="G624" t="inlineStr"/>
-      <c r="H624" t="inlineStr"/>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
@@ -21793,7 +22189,11 @@
         </is>
       </c>
       <c r="G628" t="inlineStr"/>
-      <c r="H628" t="inlineStr"/>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
@@ -21997,7 +22397,11 @@
         </is>
       </c>
       <c r="G634" t="inlineStr"/>
-      <c r="H634" t="inlineStr"/>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -22201,7 +22605,11 @@
         </is>
       </c>
       <c r="G640" t="inlineStr"/>
-      <c r="H640" t="inlineStr"/>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1on45rlaWYM</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
@@ -22235,7 +22643,11 @@
         </is>
       </c>
       <c r="G641" t="inlineStr"/>
-      <c r="H641" t="inlineStr"/>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5dDfOE8jC0c</t>
+        </is>
+      </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
@@ -22371,7 +22783,11 @@
         </is>
       </c>
       <c r="G645" t="inlineStr"/>
-      <c r="H645" t="inlineStr"/>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ajyrt6EzeLg</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
@@ -22473,7 +22889,11 @@
         </is>
       </c>
       <c r="G648" t="inlineStr"/>
-      <c r="H648" t="inlineStr"/>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
@@ -22507,7 +22927,11 @@
         </is>
       </c>
       <c r="G649" t="inlineStr"/>
-      <c r="H649" t="inlineStr"/>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
@@ -22541,7 +22965,11 @@
         </is>
       </c>
       <c r="G650" t="inlineStr"/>
-      <c r="H650" t="inlineStr"/>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
@@ -22575,7 +23003,11 @@
         </is>
       </c>
       <c r="G651" t="inlineStr"/>
-      <c r="H651" t="inlineStr"/>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
@@ -22779,7 +23211,11 @@
         </is>
       </c>
       <c r="G657" t="inlineStr"/>
-      <c r="H657" t="inlineStr"/>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
@@ -22813,7 +23249,11 @@
         </is>
       </c>
       <c r="G658" t="inlineStr"/>
-      <c r="H658" t="inlineStr"/>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
@@ -22881,7 +23321,11 @@
         </is>
       </c>
       <c r="G660" t="inlineStr"/>
-      <c r="H660" t="inlineStr"/>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -23153,7 +23597,11 @@
         </is>
       </c>
       <c r="G668" t="inlineStr"/>
-      <c r="H668" t="inlineStr"/>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr">
@@ -23255,7 +23703,11 @@
         </is>
       </c>
       <c r="G671" t="inlineStr"/>
-      <c r="H671" t="inlineStr"/>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GoiklWN9XVc</t>
+        </is>
+      </c>
     </row>
     <row r="672">
       <c r="A672" t="inlineStr">
@@ -23289,7 +23741,11 @@
         </is>
       </c>
       <c r="G672" t="inlineStr"/>
-      <c r="H672" t="inlineStr"/>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vsRJJ7z6jEI</t>
+        </is>
+      </c>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
@@ -23323,7 +23779,11 @@
         </is>
       </c>
       <c r="G673" t="inlineStr"/>
-      <c r="H673" t="inlineStr"/>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=u8Xk5GiMzkQ</t>
+        </is>
+      </c>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr">
@@ -23357,7 +23817,11 @@
         </is>
       </c>
       <c r="G674" t="inlineStr"/>
-      <c r="H674" t="inlineStr"/>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f18bLaStXVY</t>
+        </is>
+      </c>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr">
@@ -23391,7 +23855,11 @@
         </is>
       </c>
       <c r="G675" t="inlineStr"/>
-      <c r="H675" t="inlineStr"/>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7JxaSqohcNw</t>
+        </is>
+      </c>
     </row>
     <row r="676">
       <c r="A676" t="inlineStr">
@@ -23425,7 +23893,11 @@
         </is>
       </c>
       <c r="G676" t="inlineStr"/>
-      <c r="H676" t="inlineStr"/>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qNZ3dHSNkfU</t>
+        </is>
+      </c>
     </row>
     <row r="677">
       <c r="A677" t="inlineStr">
@@ -23459,7 +23931,11 @@
         </is>
       </c>
       <c r="G677" t="inlineStr"/>
-      <c r="H677" t="inlineStr"/>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="678">
       <c r="A678" t="inlineStr">
@@ -23493,7 +23969,11 @@
         </is>
       </c>
       <c r="G678" t="inlineStr"/>
-      <c r="H678" t="inlineStr"/>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="679">
       <c r="A679" t="inlineStr">
@@ -23527,7 +24007,11 @@
         </is>
       </c>
       <c r="G679" t="inlineStr"/>
-      <c r="H679" t="inlineStr"/>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="680">
       <c r="A680" t="inlineStr">
@@ -24139,7 +24623,11 @@
         </is>
       </c>
       <c r="G697" t="inlineStr"/>
-      <c r="H697" t="inlineStr"/>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-5iTx4gkHVU</t>
+        </is>
+      </c>
     </row>
     <row r="698">
       <c r="A698" t="inlineStr">
@@ -24309,7 +24797,11 @@
         </is>
       </c>
       <c r="G702" t="inlineStr"/>
-      <c r="H702" t="inlineStr"/>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wl7sjIn3cvs</t>
+        </is>
+      </c>
     </row>
     <row r="703">
       <c r="A703" t="inlineStr">
@@ -24751,7 +25243,11 @@
         </is>
       </c>
       <c r="G715" t="inlineStr"/>
-      <c r="H715" t="inlineStr"/>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=i-wl46s5bpo</t>
+        </is>
+      </c>
     </row>
     <row r="716">
       <c r="A716" t="inlineStr">
@@ -24785,7 +25281,11 @@
         </is>
       </c>
       <c r="G716" t="inlineStr"/>
-      <c r="H716" t="inlineStr"/>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9jiy7IvaDBo</t>
+        </is>
+      </c>
     </row>
     <row r="717">
       <c r="A717" t="inlineStr">
@@ -25193,7 +25693,11 @@
         </is>
       </c>
       <c r="G728" t="inlineStr"/>
-      <c r="H728" t="inlineStr"/>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=s8pED8am8KM</t>
+        </is>
+      </c>
     </row>
     <row r="729">
       <c r="A729" t="inlineStr">
@@ -25397,7 +25901,11 @@
         </is>
       </c>
       <c r="G734" t="inlineStr"/>
-      <c r="H734" t="inlineStr"/>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kAO6Z76W-Tc</t>
+        </is>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
@@ -25873,7 +26381,11 @@
         </is>
       </c>
       <c r="G748" t="inlineStr"/>
-      <c r="H748" t="inlineStr"/>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Eh6mpPfKC_U</t>
+        </is>
+      </c>
     </row>
     <row r="749">
       <c r="A749" t="inlineStr">
@@ -25907,7 +26419,11 @@
         </is>
       </c>
       <c r="G749" t="inlineStr"/>
-      <c r="H749" t="inlineStr"/>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7VdxrCrTXQM</t>
+        </is>
+      </c>
     </row>
     <row r="750">
       <c r="A750" t="inlineStr">
@@ -26417,7 +26933,11 @@
         </is>
       </c>
       <c r="G764" t="inlineStr"/>
-      <c r="H764" t="inlineStr"/>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ccN6BgtBHPA</t>
+        </is>
+      </c>
     </row>
     <row r="765">
       <c r="A765" t="inlineStr">
@@ -26451,7 +26971,11 @@
         </is>
       </c>
       <c r="G765" t="inlineStr"/>
-      <c r="H765" t="inlineStr"/>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jEW90j0xxXg</t>
+        </is>
+      </c>
     </row>
     <row r="766">
       <c r="A766" t="inlineStr">
@@ -26485,7 +27009,11 @@
         </is>
       </c>
       <c r="G766" t="inlineStr"/>
-      <c r="H766" t="inlineStr"/>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VfOWaUBln9c</t>
+        </is>
+      </c>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
@@ -26519,7 +27047,11 @@
         </is>
       </c>
       <c r="G767" t="inlineStr"/>
-      <c r="H767" t="inlineStr"/>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WJV4FCqUww8</t>
+        </is>
+      </c>
     </row>
     <row r="768">
       <c r="A768" t="inlineStr">
@@ -27029,7 +27561,11 @@
         </is>
       </c>
       <c r="G782" t="inlineStr"/>
-      <c r="H782" t="inlineStr"/>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=beNRZ7FsDQE</t>
+        </is>
+      </c>
     </row>
     <row r="783">
       <c r="A783" t="inlineStr">
@@ -27437,7 +27973,11 @@
         </is>
       </c>
       <c r="G794" t="inlineStr"/>
-      <c r="H794" t="inlineStr"/>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -27573,7 +28113,11 @@
         </is>
       </c>
       <c r="G798" t="inlineStr"/>
-      <c r="H798" t="inlineStr"/>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
@@ -27675,7 +28219,11 @@
         </is>
       </c>
       <c r="G801" t="inlineStr"/>
-      <c r="H801" t="inlineStr"/>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vHoL8JKBLCY</t>
+        </is>
+      </c>
     </row>
     <row r="802">
       <c r="A802" t="inlineStr">
@@ -27709,7 +28257,11 @@
         </is>
       </c>
       <c r="G802" t="inlineStr"/>
-      <c r="H802" t="inlineStr"/>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L_eCTqzS4EY</t>
+        </is>
+      </c>
     </row>
     <row r="803">
       <c r="A803" t="inlineStr">
@@ -27913,7 +28465,11 @@
         </is>
       </c>
       <c r="G808" t="inlineStr"/>
-      <c r="H808" t="inlineStr"/>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ccITevjFTrQ</t>
+        </is>
+      </c>
     </row>
     <row r="809">
       <c r="A809" t="inlineStr">
@@ -27947,7 +28503,11 @@
         </is>
       </c>
       <c r="G809" t="inlineStr"/>
-      <c r="H809" t="inlineStr"/>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=40UUr4vRX7g</t>
+        </is>
+      </c>
     </row>
     <row r="810">
       <c r="A810" t="inlineStr">
@@ -28185,7 +28745,11 @@
         </is>
       </c>
       <c r="G816" t="inlineStr"/>
-      <c r="H816" t="inlineStr"/>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=40UUr4vRX7g</t>
+        </is>
+      </c>
     </row>
     <row r="817">
       <c r="A817" t="inlineStr">
@@ -28219,7 +28783,11 @@
         </is>
       </c>
       <c r="G817" t="inlineStr"/>
-      <c r="H817" t="inlineStr"/>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=40UUr4vRX7g</t>
+        </is>
+      </c>
     </row>
     <row r="818">
       <c r="A818" t="inlineStr">
@@ -28287,7 +28855,11 @@
         </is>
       </c>
       <c r="G819" t="inlineStr"/>
-      <c r="H819" t="inlineStr"/>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr">
@@ -28423,7 +28995,11 @@
         </is>
       </c>
       <c r="G823" t="inlineStr"/>
-      <c r="H823" t="inlineStr"/>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0m5s6BWrPg8</t>
+        </is>
+      </c>
     </row>
     <row r="824">
       <c r="A824" t="inlineStr">
@@ -28661,7 +29237,11 @@
         </is>
       </c>
       <c r="G830" t="inlineStr"/>
-      <c r="H830" t="inlineStr"/>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HJVjFmaU61g</t>
+        </is>
+      </c>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr">
@@ -28797,7 +29377,11 @@
         </is>
       </c>
       <c r="G834" t="inlineStr"/>
-      <c r="H834" t="inlineStr"/>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HJVjFmaU61g</t>
+        </is>
+      </c>
     </row>
     <row r="835">
       <c r="A835" t="inlineStr">
@@ -29103,7 +29687,11 @@
         </is>
       </c>
       <c r="G843" t="inlineStr"/>
-      <c r="H843" t="inlineStr"/>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1sCvnCEFLqg</t>
+        </is>
+      </c>
     </row>
     <row r="844">
       <c r="A844" t="inlineStr">
@@ -29137,7 +29725,11 @@
         </is>
       </c>
       <c r="G844" t="inlineStr"/>
-      <c r="H844" t="inlineStr"/>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1sCvnCEFLqg</t>
+        </is>
+      </c>
     </row>
     <row r="845">
       <c r="A845" t="inlineStr">
@@ -29171,7 +29763,11 @@
         </is>
       </c>
       <c r="G845" t="inlineStr"/>
-      <c r="H845" t="inlineStr"/>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1sCvnCEFLqg</t>
+        </is>
+      </c>
     </row>
     <row r="846">
       <c r="A846" t="inlineStr">
@@ -29205,7 +29801,11 @@
         </is>
       </c>
       <c r="G846" t="inlineStr"/>
-      <c r="H846" t="inlineStr"/>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1sCvnCEFLqg</t>
+        </is>
+      </c>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
@@ -29341,7 +29941,11 @@
         </is>
       </c>
       <c r="G850" t="inlineStr"/>
-      <c r="H850" t="inlineStr"/>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="851">
       <c r="A851" t="inlineStr">
@@ -29579,7 +30183,11 @@
         </is>
       </c>
       <c r="G857" t="inlineStr"/>
-      <c r="H857" t="inlineStr"/>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="858">
       <c r="A858" t="inlineStr">
@@ -30191,7 +30799,11 @@
         </is>
       </c>
       <c r="G875" t="inlineStr"/>
-      <c r="H875" t="inlineStr"/>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Pc460WNyeeI</t>
+        </is>
+      </c>
     </row>
     <row r="876">
       <c r="A876" t="inlineStr">
@@ -30225,7 +30837,11 @@
         </is>
       </c>
       <c r="G876" t="inlineStr"/>
-      <c r="H876" t="inlineStr"/>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JQpEwQSzVhM</t>
+        </is>
+      </c>
     </row>
     <row r="877">
       <c r="A877" t="inlineStr">
@@ -30259,7 +30875,11 @@
         </is>
       </c>
       <c r="G877" t="inlineStr"/>
-      <c r="H877" t="inlineStr"/>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Xlokhrhq4QI</t>
+        </is>
+      </c>
     </row>
     <row r="878">
       <c r="A878" t="inlineStr">
@@ -30735,7 +31355,11 @@
         </is>
       </c>
       <c r="G891" t="inlineStr"/>
-      <c r="H891" t="inlineStr"/>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0QUgsmRP9Eo</t>
+        </is>
+      </c>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
@@ -30769,7 +31393,11 @@
         </is>
       </c>
       <c r="G892" t="inlineStr"/>
-      <c r="H892" t="inlineStr"/>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MIxSzBWgsrI</t>
+        </is>
+      </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
@@ -30803,7 +31431,11 @@
         </is>
       </c>
       <c r="G893" t="inlineStr"/>
-      <c r="H893" t="inlineStr"/>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zQCtlp4q800</t>
+        </is>
+      </c>
     </row>
     <row r="894">
       <c r="A894" t="inlineStr">
@@ -30837,7 +31469,11 @@
         </is>
       </c>
       <c r="G894" t="inlineStr"/>
-      <c r="H894" t="inlineStr"/>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dgQFdX4pAZA</t>
+        </is>
+      </c>
     </row>
     <row r="895">
       <c r="A895" t="inlineStr">
@@ -30871,7 +31507,11 @@
         </is>
       </c>
       <c r="G895" t="inlineStr"/>
-      <c r="H895" t="inlineStr"/>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4DPtF9vKiI</t>
+        </is>
+      </c>
     </row>
     <row r="896">
       <c r="A896" t="inlineStr">
@@ -30905,7 +31545,11 @@
         </is>
       </c>
       <c r="G896" t="inlineStr"/>
-      <c r="H896" t="inlineStr"/>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pwc964xKO-w</t>
+        </is>
+      </c>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
@@ -30939,7 +31583,11 @@
         </is>
       </c>
       <c r="G897" t="inlineStr"/>
-      <c r="H897" t="inlineStr"/>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CPrMHajxyAw</t>
+        </is>
+      </c>
     </row>
     <row r="898">
       <c r="A898" t="inlineStr">
@@ -30973,7 +31621,11 @@
         </is>
       </c>
       <c r="G898" t="inlineStr"/>
-      <c r="H898" t="inlineStr"/>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Wvjsb6ZVcHA</t>
+        </is>
+      </c>
     </row>
     <row r="899">
       <c r="A899" t="inlineStr">
@@ -31007,7 +31659,11 @@
         </is>
       </c>
       <c r="G899" t="inlineStr"/>
-      <c r="H899" t="inlineStr"/>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TyoVQN9d0hM</t>
+        </is>
+      </c>
     </row>
     <row r="900">
       <c r="A900" t="inlineStr">
@@ -31041,7 +31697,11 @@
         </is>
       </c>
       <c r="G900" t="inlineStr"/>
-      <c r="H900" t="inlineStr"/>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1ipqho4OlhI</t>
+        </is>
+      </c>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
@@ -31075,7 +31735,11 @@
         </is>
       </c>
       <c r="G901" t="inlineStr"/>
-      <c r="H901" t="inlineStr"/>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=v-rDLzzdcvg</t>
+        </is>
+      </c>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
@@ -31109,7 +31773,11 @@
         </is>
       </c>
       <c r="G902" t="inlineStr"/>
-      <c r="H902" t="inlineStr"/>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=E9hDWUueNuo</t>
+        </is>
+      </c>
     </row>
     <row r="903">
       <c r="A903" t="inlineStr">
@@ -31143,7 +31811,11 @@
         </is>
       </c>
       <c r="G903" t="inlineStr"/>
-      <c r="H903" t="inlineStr"/>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-QPklG6E2s8</t>
+        </is>
+      </c>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -31177,7 +31849,11 @@
         </is>
       </c>
       <c r="G904" t="inlineStr"/>
-      <c r="H904" t="inlineStr"/>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fHWWxthzHWE</t>
+        </is>
+      </c>
     </row>
     <row r="905">
       <c r="A905" t="inlineStr">
@@ -31211,7 +31887,11 @@
         </is>
       </c>
       <c r="G905" t="inlineStr"/>
-      <c r="H905" t="inlineStr"/>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eHE6NhwU8JU</t>
+        </is>
+      </c>
     </row>
     <row r="906">
       <c r="A906" t="inlineStr">
@@ -31245,7 +31925,11 @@
         </is>
       </c>
       <c r="G906" t="inlineStr"/>
-      <c r="H906" t="inlineStr"/>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=q1rBTxUgpoU</t>
+        </is>
+      </c>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">
@@ -31279,7 +31963,11 @@
         </is>
       </c>
       <c r="G907" t="inlineStr"/>
-      <c r="H907" t="inlineStr"/>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6WHf8iq27zU</t>
+        </is>
+      </c>
     </row>
     <row r="908">
       <c r="A908" t="inlineStr">
@@ -31313,7 +32001,11 @@
         </is>
       </c>
       <c r="G908" t="inlineStr"/>
-      <c r="H908" t="inlineStr"/>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J6TjB20x7zU</t>
+        </is>
+      </c>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
@@ -31347,7 +32039,11 @@
         </is>
       </c>
       <c r="G909" t="inlineStr"/>
-      <c r="H909" t="inlineStr"/>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mqfU3s74jCA</t>
+        </is>
+      </c>
     </row>
     <row r="910">
       <c r="A910" t="inlineStr">
@@ -31381,7 +32077,11 @@
         </is>
       </c>
       <c r="G910" t="inlineStr"/>
-      <c r="H910" t="inlineStr"/>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mUqZo7nGFf4</t>
+        </is>
+      </c>
     </row>
     <row r="911">
       <c r="A911" t="inlineStr">
@@ -31415,7 +32115,11 @@
         </is>
       </c>
       <c r="G911" t="inlineStr"/>
-      <c r="H911" t="inlineStr"/>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eWgIU2MHXDM</t>
+        </is>
+      </c>
     </row>
     <row r="912">
       <c r="A912" t="inlineStr">
@@ -31449,7 +32153,11 @@
         </is>
       </c>
       <c r="G912" t="inlineStr"/>
-      <c r="H912" t="inlineStr"/>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Uv3KiJU-Wdo</t>
+        </is>
+      </c>
     </row>
     <row r="913">
       <c r="A913" t="inlineStr">
@@ -31483,7 +32191,11 @@
         </is>
       </c>
       <c r="G913" t="inlineStr"/>
-      <c r="H913" t="inlineStr"/>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=giQdRZVPGMM</t>
+        </is>
+      </c>
     </row>
     <row r="914">
       <c r="A914" t="inlineStr">
@@ -31551,7 +32263,11 @@
         </is>
       </c>
       <c r="G915" t="inlineStr"/>
-      <c r="H915" t="inlineStr"/>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vBp-A46Pqhs</t>
+        </is>
+      </c>
     </row>
     <row r="916">
       <c r="A916" t="inlineStr">
@@ -31585,7 +32301,11 @@
         </is>
       </c>
       <c r="G916" t="inlineStr"/>
-      <c r="H916" t="inlineStr"/>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SvuyoZ8dGpU</t>
+        </is>
+      </c>
     </row>
     <row r="917">
       <c r="A917" t="inlineStr">
@@ -31619,7 +32339,11 @@
         </is>
       </c>
       <c r="G917" t="inlineStr"/>
-      <c r="H917" t="inlineStr"/>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GhxVQtpG6V0</t>
+        </is>
+      </c>
     </row>
     <row r="918">
       <c r="A918" t="inlineStr">
@@ -31653,7 +32377,11 @@
         </is>
       </c>
       <c r="G918" t="inlineStr"/>
-      <c r="H918" t="inlineStr"/>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0Z4xjEij2jo</t>
+        </is>
+      </c>
     </row>
     <row r="919">
       <c r="A919" t="inlineStr">
@@ -31687,7 +32415,11 @@
         </is>
       </c>
       <c r="G919" t="inlineStr"/>
-      <c r="H919" t="inlineStr"/>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ucsedtlKMSs</t>
+        </is>
+      </c>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
@@ -31721,7 +32453,11 @@
         </is>
       </c>
       <c r="G920" t="inlineStr"/>
-      <c r="H920" t="inlineStr"/>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Ap5n5y88ZAY</t>
+        </is>
+      </c>
     </row>
     <row r="921">
       <c r="A921" t="inlineStr">
@@ -31755,7 +32491,11 @@
         </is>
       </c>
       <c r="G921" t="inlineStr"/>
-      <c r="H921" t="inlineStr"/>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qHSBWEE5Ycg</t>
+        </is>
+      </c>
     </row>
     <row r="922">
       <c r="A922" t="inlineStr">
@@ -31789,7 +32529,11 @@
         </is>
       </c>
       <c r="G922" t="inlineStr"/>
-      <c r="H922" t="inlineStr"/>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1N53mPAsEy0</t>
+        </is>
+      </c>
     </row>
     <row r="923">
       <c r="A923" t="inlineStr">
@@ -31823,7 +32567,11 @@
         </is>
       </c>
       <c r="G923" t="inlineStr"/>
-      <c r="H923" t="inlineStr"/>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BjdETsv7AEI</t>
+        </is>
+      </c>
     </row>
     <row r="924">
       <c r="A924" t="inlineStr">
@@ -31857,7 +32605,11 @@
         </is>
       </c>
       <c r="G924" t="inlineStr"/>
-      <c r="H924" t="inlineStr"/>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZaDvfiXhqvI</t>
+        </is>
+      </c>
     </row>
     <row r="925">
       <c r="A925" t="inlineStr">
@@ -31891,7 +32643,11 @@
         </is>
       </c>
       <c r="G925" t="inlineStr"/>
-      <c r="H925" t="inlineStr"/>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=DPgnp1XNT0A</t>
+        </is>
+      </c>
     </row>
     <row r="926">
       <c r="A926" t="inlineStr">
@@ -31925,7 +32681,11 @@
         </is>
       </c>
       <c r="G926" t="inlineStr"/>
-      <c r="H926" t="inlineStr"/>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GM3IWrpcSm4</t>
+        </is>
+      </c>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">
@@ -31959,7 +32719,11 @@
         </is>
       </c>
       <c r="G927" t="inlineStr"/>
-      <c r="H927" t="inlineStr"/>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jUF8A5kISkk</t>
+        </is>
+      </c>
     </row>
     <row r="928">
       <c r="A928" t="inlineStr">
@@ -31993,7 +32757,11 @@
         </is>
       </c>
       <c r="G928" t="inlineStr"/>
-      <c r="H928" t="inlineStr"/>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FUIFYyQisTA</t>
+        </is>
+      </c>
     </row>
     <row r="929">
       <c r="A929" t="inlineStr">
@@ -32027,7 +32795,11 @@
         </is>
       </c>
       <c r="G929" t="inlineStr"/>
-      <c r="H929" t="inlineStr"/>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=c5ilsh3p5lM</t>
+        </is>
+      </c>
     </row>
     <row r="930">
       <c r="A930" t="inlineStr">
@@ -32061,7 +32833,11 @@
         </is>
       </c>
       <c r="G930" t="inlineStr"/>
-      <c r="H930" t="inlineStr"/>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FZGcvVok2s8</t>
+        </is>
+      </c>
     </row>
     <row r="931">
       <c r="A931" t="inlineStr">
@@ -32095,7 +32871,11 @@
         </is>
       </c>
       <c r="G931" t="inlineStr"/>
-      <c r="H931" t="inlineStr"/>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FZGcvVok2s8</t>
+        </is>
+      </c>
     </row>
     <row r="932">
       <c r="A932" t="inlineStr">
@@ -32129,7 +32909,11 @@
         </is>
       </c>
       <c r="G932" t="inlineStr"/>
-      <c r="H932" t="inlineStr"/>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FZGcvVok2s8</t>
+        </is>
+      </c>
     </row>
     <row r="933">
       <c r="A933" t="inlineStr">
@@ -32163,7 +32947,11 @@
         </is>
       </c>
       <c r="G933" t="inlineStr"/>
-      <c r="H933" t="inlineStr"/>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=juIcoqpy0UM</t>
+        </is>
+      </c>
     </row>
     <row r="934">
       <c r="A934" t="inlineStr">
@@ -32197,7 +32985,11 @@
         </is>
       </c>
       <c r="G934" t="inlineStr"/>
-      <c r="H934" t="inlineStr"/>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GUKH-2zRBfo</t>
+        </is>
+      </c>
     </row>
     <row r="935">
       <c r="A935" t="inlineStr">
@@ -32231,7 +33023,11 @@
         </is>
       </c>
       <c r="G935" t="inlineStr"/>
-      <c r="H935" t="inlineStr"/>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Bua4ksLkc_I</t>
+        </is>
+      </c>
     </row>
     <row r="936">
       <c r="A936" t="inlineStr">
@@ -37567,7 +38363,11 @@
         </is>
       </c>
       <c r="G1087" t="inlineStr"/>
-      <c r="H1087" t="inlineStr"/>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kLotjCnlBjA</t>
+        </is>
+      </c>
     </row>
     <row r="1088">
       <c r="A1088" t="inlineStr">
@@ -37749,7 +38549,11 @@
         </is>
       </c>
       <c r="G1092" t="inlineStr"/>
-      <c r="H1092" t="inlineStr"/>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6I-3A99mc9s</t>
+        </is>
+      </c>
     </row>
     <row r="1093">
       <c r="A1093" t="inlineStr">
@@ -37821,7 +38625,11 @@
         </is>
       </c>
       <c r="G1094" t="inlineStr"/>
-      <c r="H1094" t="inlineStr"/>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wXDEAQyF7oU</t>
+        </is>
+      </c>
     </row>
     <row r="1095">
       <c r="A1095" t="inlineStr">
@@ -37893,7 +38701,11 @@
         </is>
       </c>
       <c r="G1096" t="inlineStr"/>
-      <c r="H1096" t="inlineStr"/>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TrrQzz4IjXk</t>
+        </is>
+      </c>
     </row>
     <row r="1097">
       <c r="A1097" t="inlineStr">
@@ -38185,7 +38997,11 @@
         </is>
       </c>
       <c r="G1104" t="inlineStr"/>
-      <c r="H1104" t="inlineStr"/>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XcePRTr8ibE</t>
+        </is>
+      </c>
     </row>
     <row r="1105">
       <c r="A1105" t="inlineStr">
@@ -38321,7 +39137,11 @@
         </is>
       </c>
       <c r="G1108" t="inlineStr"/>
-      <c r="H1108" t="inlineStr"/>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3UYLbzYEnDE</t>
+        </is>
+      </c>
     </row>
     <row r="1109">
       <c r="A1109" t="inlineStr">
@@ -38355,7 +39175,11 @@
         </is>
       </c>
       <c r="G1109" t="inlineStr"/>
-      <c r="H1109" t="inlineStr"/>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5ocqLPfI82M</t>
+        </is>
+      </c>
     </row>
     <row r="1110">
       <c r="A1110" t="inlineStr">
@@ -38389,7 +39213,11 @@
         </is>
       </c>
       <c r="G1110" t="inlineStr"/>
-      <c r="H1110" t="inlineStr"/>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=apK9Zlp_VuQ</t>
+        </is>
+      </c>
     </row>
     <row r="1111">
       <c r="A1111" t="inlineStr">
@@ -38423,7 +39251,11 @@
         </is>
       </c>
       <c r="G1111" t="inlineStr"/>
-      <c r="H1111" t="inlineStr"/>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1WL6cLE-PKI</t>
+        </is>
+      </c>
     </row>
     <row r="1112">
       <c r="A1112" t="inlineStr">
@@ -38457,7 +39289,11 @@
         </is>
       </c>
       <c r="G1112" t="inlineStr"/>
-      <c r="H1112" t="inlineStr"/>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MGsFGIefdME</t>
+        </is>
+      </c>
     </row>
     <row r="1113">
       <c r="A1113" t="inlineStr">
@@ -38491,7 +39327,11 @@
         </is>
       </c>
       <c r="G1113" t="inlineStr"/>
-      <c r="H1113" t="inlineStr"/>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3UYLbzYEnDE</t>
+        </is>
+      </c>
     </row>
     <row r="1114">
       <c r="A1114" t="inlineStr">
@@ -38745,7 +39585,11 @@
         </is>
       </c>
       <c r="G1120" t="inlineStr"/>
-      <c r="H1120" t="inlineStr"/>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yStexJD70po</t>
+        </is>
+      </c>
     </row>
     <row r="1121">
       <c r="A1121" t="inlineStr">
@@ -38893,7 +39737,11 @@
         </is>
       </c>
       <c r="G1124" t="inlineStr"/>
-      <c r="H1124" t="inlineStr"/>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J8YFuqa6tEU</t>
+        </is>
+      </c>
     </row>
     <row r="1125">
       <c r="A1125" t="inlineStr">
@@ -38927,7 +39775,11 @@
         </is>
       </c>
       <c r="G1125" t="inlineStr"/>
-      <c r="H1125" t="inlineStr"/>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J8YFuqa6tEU</t>
+        </is>
+      </c>
     </row>
     <row r="1126">
       <c r="A1126" t="inlineStr">
@@ -38961,7 +39813,11 @@
         </is>
       </c>
       <c r="G1126" t="inlineStr"/>
-      <c r="H1126" t="inlineStr"/>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J8YFuqa6tEU</t>
+        </is>
+      </c>
     </row>
     <row r="1127">
       <c r="A1127" t="inlineStr">
@@ -39185,7 +40041,11 @@
         </is>
       </c>
       <c r="G1132" t="inlineStr"/>
-      <c r="H1132" t="inlineStr"/>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gKVyjWEIIno</t>
+        </is>
+      </c>
     </row>
     <row r="1133">
       <c r="A1133" t="inlineStr">
@@ -39219,7 +40079,11 @@
         </is>
       </c>
       <c r="G1133" t="inlineStr"/>
-      <c r="H1133" t="inlineStr"/>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rSptuCSPRxE</t>
+        </is>
+      </c>
     </row>
     <row r="1134">
       <c r="A1134" t="inlineStr">
@@ -39253,7 +40117,11 @@
         </is>
       </c>
       <c r="G1134" t="inlineStr"/>
-      <c r="H1134" t="inlineStr"/>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gKVyjWEIIno</t>
+        </is>
+      </c>
     </row>
     <row r="1135">
       <c r="A1135" t="inlineStr">
@@ -39515,7 +40383,11 @@
         </is>
       </c>
       <c r="G1141" t="inlineStr"/>
-      <c r="H1141" t="inlineStr"/>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k24UAsSiY14</t>
+        </is>
+      </c>
     </row>
     <row r="1142">
       <c r="A1142" t="inlineStr">
@@ -39587,7 +40459,11 @@
         </is>
       </c>
       <c r="G1143" t="inlineStr"/>
-      <c r="H1143" t="inlineStr"/>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_ZqYHMoJ_-w</t>
+        </is>
+      </c>
     </row>
     <row r="1144">
       <c r="A1144" t="inlineStr">
@@ -39621,7 +40497,11 @@
         </is>
       </c>
       <c r="G1144" t="inlineStr"/>
-      <c r="H1144" t="inlineStr"/>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MBMFuPjFw7E</t>
+        </is>
+      </c>
     </row>
     <row r="1145">
       <c r="A1145" t="inlineStr">
@@ -39655,7 +40535,11 @@
         </is>
       </c>
       <c r="G1145" t="inlineStr"/>
-      <c r="H1145" t="inlineStr"/>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=voAh9e9MAJA</t>
+        </is>
+      </c>
     </row>
     <row r="1146">
       <c r="A1146" t="inlineStr">
@@ -39689,7 +40573,11 @@
         </is>
       </c>
       <c r="G1146" t="inlineStr"/>
-      <c r="H1146" t="inlineStr"/>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ScS30T755BE</t>
+        </is>
+      </c>
     </row>
     <row r="1147">
       <c r="A1147" t="inlineStr">
@@ -39871,7 +40759,11 @@
         </is>
       </c>
       <c r="G1151" t="inlineStr"/>
-      <c r="H1151" t="inlineStr"/>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R6CKf72ZcmE</t>
+        </is>
+      </c>
     </row>
     <row r="1152">
       <c r="A1152" t="inlineStr">
@@ -39905,7 +40797,11 @@
         </is>
       </c>
       <c r="G1152" t="inlineStr"/>
-      <c r="H1152" t="inlineStr"/>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R6CKf72ZcmE</t>
+        </is>
+      </c>
     </row>
     <row r="1153">
       <c r="A1153" t="inlineStr">
@@ -39939,7 +40835,11 @@
         </is>
       </c>
       <c r="G1153" t="inlineStr"/>
-      <c r="H1153" t="inlineStr"/>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R6CKf72ZcmE</t>
+        </is>
+      </c>
     </row>
     <row r="1154">
       <c r="A1154" t="inlineStr">
@@ -39973,7 +40873,11 @@
         </is>
       </c>
       <c r="G1154" t="inlineStr"/>
-      <c r="H1154" t="inlineStr"/>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R6CKf72ZcmE</t>
+        </is>
+      </c>
     </row>
     <row r="1155">
       <c r="A1155" t="inlineStr">
@@ -40113,7 +41017,11 @@
         </is>
       </c>
       <c r="G1158" t="inlineStr"/>
-      <c r="H1158" t="inlineStr"/>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zwsMP0dSjmY</t>
+        </is>
+      </c>
     </row>
     <row r="1159">
       <c r="A1159" t="inlineStr">
@@ -40147,7 +41055,11 @@
         </is>
       </c>
       <c r="G1159" t="inlineStr"/>
-      <c r="H1159" t="inlineStr"/>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zwsMP0dSjmY</t>
+        </is>
+      </c>
     </row>
     <row r="1160">
       <c r="A1160" t="inlineStr">
@@ -40389,7 +41301,11 @@
         </is>
       </c>
       <c r="G1166" t="inlineStr"/>
-      <c r="H1166" t="inlineStr"/>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=q3BrCmbJSA4</t>
+        </is>
+      </c>
     </row>
     <row r="1167">
       <c r="A1167" t="inlineStr">
@@ -40457,7 +41373,11 @@
         </is>
       </c>
       <c r="G1168" t="inlineStr"/>
-      <c r="H1168" t="inlineStr"/>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6jY-ljzRsbg</t>
+        </is>
+      </c>
     </row>
     <row r="1169">
       <c r="A1169" t="inlineStr">
@@ -40491,7 +41411,11 @@
         </is>
       </c>
       <c r="G1169" t="inlineStr"/>
-      <c r="H1169" t="inlineStr"/>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4oOHYuLYZ7A</t>
+        </is>
+      </c>
     </row>
     <row r="1170">
       <c r="A1170" t="inlineStr">
@@ -40559,7 +41483,11 @@
         </is>
       </c>
       <c r="G1171" t="inlineStr"/>
-      <c r="H1171" t="inlineStr"/>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tEv5mPKoHjA</t>
+        </is>
+      </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
@@ -40627,7 +41555,11 @@
         </is>
       </c>
       <c r="G1173" t="inlineStr"/>
-      <c r="H1173" t="inlineStr"/>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4oOHYuLYZ7A</t>
+        </is>
+      </c>
     </row>
     <row r="1174">
       <c r="A1174" t="inlineStr">
@@ -40797,7 +41729,11 @@
         </is>
       </c>
       <c r="G1178" t="inlineStr"/>
-      <c r="H1178" t="inlineStr"/>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2YgUNGEQ8J0</t>
+        </is>
+      </c>
     </row>
     <row r="1179">
       <c r="A1179" t="inlineStr">
@@ -40907,7 +41843,11 @@
         </is>
       </c>
       <c r="G1181" t="inlineStr"/>
-      <c r="H1181" t="inlineStr"/>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2YgUNGEQ8J0</t>
+        </is>
+      </c>
     </row>
     <row r="1182">
       <c r="A1182" t="inlineStr">
@@ -40941,7 +41881,11 @@
         </is>
       </c>
       <c r="G1182" t="inlineStr"/>
-      <c r="H1182" t="inlineStr"/>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2YgUNGEQ8J0</t>
+        </is>
+      </c>
     </row>
     <row r="1183">
       <c r="A1183" t="inlineStr">
@@ -40975,7 +41919,11 @@
         </is>
       </c>
       <c r="G1183" t="inlineStr"/>
-      <c r="H1183" t="inlineStr"/>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2YgUNGEQ8J0</t>
+        </is>
+      </c>
     </row>
     <row r="1184">
       <c r="A1184" t="inlineStr">
@@ -41417,7 +42365,11 @@
         </is>
       </c>
       <c r="G1196" t="inlineStr"/>
-      <c r="H1196" t="inlineStr"/>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gL6jMezAhR4</t>
+        </is>
+      </c>
     </row>
     <row r="1197">
       <c r="A1197" t="inlineStr">
@@ -41451,7 +42403,11 @@
         </is>
       </c>
       <c r="G1197" t="inlineStr"/>
-      <c r="H1197" t="inlineStr"/>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=DQFHyjea844</t>
+        </is>
+      </c>
     </row>
     <row r="1198">
       <c r="A1198" t="inlineStr">
@@ -41485,7 +42441,11 @@
         </is>
       </c>
       <c r="G1198" t="inlineStr"/>
-      <c r="H1198" t="inlineStr"/>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gL6jMezAhR4</t>
+        </is>
+      </c>
     </row>
     <row r="1199">
       <c r="A1199" t="inlineStr">
@@ -41519,7 +42479,11 @@
         </is>
       </c>
       <c r="G1199" t="inlineStr"/>
-      <c r="H1199" t="inlineStr"/>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gL6jMezAhR4</t>
+        </is>
+      </c>
     </row>
     <row r="1200">
       <c r="A1200" t="inlineStr">
@@ -41553,7 +42517,11 @@
         </is>
       </c>
       <c r="G1200" t="inlineStr"/>
-      <c r="H1200" t="inlineStr"/>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bT_uZ5l6pL0</t>
+        </is>
+      </c>
     </row>
     <row r="1201">
       <c r="A1201" t="inlineStr">
@@ -41587,7 +42555,11 @@
         </is>
       </c>
       <c r="G1201" t="inlineStr"/>
-      <c r="H1201" t="inlineStr"/>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bT_uZ5l6pL0</t>
+        </is>
+      </c>
     </row>
     <row r="1202">
       <c r="A1202" t="inlineStr">
@@ -41621,7 +42593,11 @@
         </is>
       </c>
       <c r="G1202" t="inlineStr"/>
-      <c r="H1202" t="inlineStr"/>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=b2BxXCjTG7A</t>
+        </is>
+      </c>
     </row>
     <row r="1203">
       <c r="A1203" t="inlineStr">
@@ -41655,7 +42631,11 @@
         </is>
       </c>
       <c r="G1203" t="inlineStr"/>
-      <c r="H1203" t="inlineStr"/>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gL6jMezAhR4</t>
+        </is>
+      </c>
     </row>
     <row r="1204">
       <c r="A1204" t="inlineStr">
@@ -41689,7 +42669,11 @@
         </is>
       </c>
       <c r="G1204" t="inlineStr"/>
-      <c r="H1204" t="inlineStr"/>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=b2BxXCjTG7A</t>
+        </is>
+      </c>
     </row>
     <row r="1205">
       <c r="A1205" t="inlineStr">
@@ -42041,7 +43025,11 @@
         </is>
       </c>
       <c r="G1214" t="inlineStr"/>
-      <c r="H1214" t="inlineStr"/>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=70qHuU4lMU0</t>
+        </is>
+      </c>
     </row>
     <row r="1215">
       <c r="A1215" t="inlineStr">
@@ -42075,7 +43063,11 @@
         </is>
       </c>
       <c r="G1215" t="inlineStr"/>
-      <c r="H1215" t="inlineStr"/>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sUb8wg528lU</t>
+        </is>
+      </c>
     </row>
     <row r="1216">
       <c r="A1216" t="inlineStr">
@@ -42181,7 +43173,11 @@
         </is>
       </c>
       <c r="G1218" t="inlineStr"/>
-      <c r="H1218" t="inlineStr"/>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GdPj5ppmz5Y</t>
+        </is>
+      </c>
     </row>
     <row r="1219">
       <c r="A1219" t="inlineStr">
@@ -42253,7 +43249,11 @@
         </is>
       </c>
       <c r="G1220" t="inlineStr"/>
-      <c r="H1220" t="inlineStr"/>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GdPj5ppmz5Y</t>
+        </is>
+      </c>
     </row>
     <row r="1221">
       <c r="A1221" t="inlineStr">
@@ -42287,7 +43287,11 @@
         </is>
       </c>
       <c r="G1221" t="inlineStr"/>
-      <c r="H1221" t="inlineStr"/>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=UUjDBIKwRnQ</t>
+        </is>
+      </c>
     </row>
     <row r="1222">
       <c r="A1222" t="inlineStr">
@@ -42389,7 +43393,11 @@
         </is>
       </c>
       <c r="G1224" t="inlineStr"/>
-      <c r="H1224" t="inlineStr"/>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HMVEP73WGLs</t>
+        </is>
+      </c>
     </row>
     <row r="1225">
       <c r="A1225" t="inlineStr">
@@ -42457,7 +43465,11 @@
         </is>
       </c>
       <c r="G1226" t="inlineStr"/>
-      <c r="H1226" t="inlineStr"/>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=o-fux1zma70</t>
+        </is>
+      </c>
     </row>
     <row r="1227">
       <c r="A1227" t="inlineStr">
@@ -42491,7 +43503,11 @@
         </is>
       </c>
       <c r="G1227" t="inlineStr"/>
-      <c r="H1227" t="inlineStr"/>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=o-fux1zma70</t>
+        </is>
+      </c>
     </row>
     <row r="1228">
       <c r="A1228" t="inlineStr">
@@ -42525,7 +43541,11 @@
         </is>
       </c>
       <c r="G1228" t="inlineStr"/>
-      <c r="H1228" t="inlineStr"/>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=o-fux1zma70</t>
+        </is>
+      </c>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
@@ -42559,7 +43579,11 @@
         </is>
       </c>
       <c r="G1229" t="inlineStr"/>
-      <c r="H1229" t="inlineStr"/>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M-fYYECjNq0</t>
+        </is>
+      </c>
     </row>
     <row r="1230">
       <c r="A1230" t="inlineStr">
@@ -42593,7 +43617,11 @@
         </is>
       </c>
       <c r="G1230" t="inlineStr"/>
-      <c r="H1230" t="inlineStr"/>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M-fYYECjNq0</t>
+        </is>
+      </c>
     </row>
     <row r="1231">
       <c r="A1231" t="inlineStr">
@@ -42627,7 +43655,11 @@
         </is>
       </c>
       <c r="G1231" t="inlineStr"/>
-      <c r="H1231" t="inlineStr"/>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YHLbYR8YZys</t>
+        </is>
+      </c>
     </row>
     <row r="1232">
       <c r="A1232" t="inlineStr">
@@ -42661,7 +43693,11 @@
         </is>
       </c>
       <c r="G1232" t="inlineStr"/>
-      <c r="H1232" t="inlineStr"/>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YHLbYR8YZys</t>
+        </is>
+      </c>
     </row>
     <row r="1233">
       <c r="A1233" t="inlineStr">
@@ -42695,7 +43731,11 @@
         </is>
       </c>
       <c r="G1233" t="inlineStr"/>
-      <c r="H1233" t="inlineStr"/>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rORrRAnD1no</t>
+        </is>
+      </c>
     </row>
     <row r="1234">
       <c r="A1234" t="inlineStr">
@@ -42729,7 +43769,11 @@
         </is>
       </c>
       <c r="G1234" t="inlineStr"/>
-      <c r="H1234" t="inlineStr"/>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rORrRAnD1no</t>
+        </is>
+      </c>
     </row>
     <row r="1235">
       <c r="A1235" t="inlineStr">
@@ -42801,7 +43845,11 @@
           <t>https://www.imex.cl/fichas/BLSG7LBLIS02.pdf</t>
         </is>
       </c>
-      <c r="H1236" t="inlineStr"/>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1237">
       <c r="A1237" t="inlineStr">
@@ -42835,7 +43883,11 @@
         </is>
       </c>
       <c r="G1237" t="inlineStr"/>
-      <c r="H1237" t="inlineStr"/>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1238">
       <c r="A1238" t="inlineStr">
@@ -42873,7 +43925,11 @@
           <t>https://www.imex.cl/fichas/BLSG7BBLIS01.pdf</t>
         </is>
       </c>
-      <c r="H1238" t="inlineStr"/>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
@@ -42907,7 +43963,11 @@
         </is>
       </c>
       <c r="G1239" t="inlineStr"/>
-      <c r="H1239" t="inlineStr"/>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f5s7O9b7M1g</t>
+        </is>
+      </c>
     </row>
     <row r="1240">
       <c r="A1240" t="inlineStr">
@@ -42941,7 +44001,11 @@
         </is>
       </c>
       <c r="G1240" t="inlineStr"/>
-      <c r="H1240" t="inlineStr"/>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f5s7O9b7M1g</t>
+        </is>
+      </c>
     </row>
     <row r="1241">
       <c r="A1241" t="inlineStr">
@@ -42975,7 +44039,11 @@
         </is>
       </c>
       <c r="G1241" t="inlineStr"/>
-      <c r="H1241" t="inlineStr"/>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5WwK192kiSw</t>
+        </is>
+      </c>
     </row>
     <row r="1242">
       <c r="A1242" t="inlineStr">
@@ -43013,7 +44081,11 @@
           <t>https://www.imex.cl/fichas/SWPTBR.pdf</t>
         </is>
       </c>
-      <c r="H1242" t="inlineStr"/>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1243">
       <c r="A1243" t="inlineStr">
@@ -43051,7 +44123,11 @@
           <t>https://www.imex.cl/fichas/SWPTBLG.pdf</t>
         </is>
       </c>
-      <c r="H1243" t="inlineStr"/>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1244">
       <c r="A1244" t="inlineStr">
@@ -43085,7 +44161,11 @@
         </is>
       </c>
       <c r="G1244" t="inlineStr"/>
-      <c r="H1244" t="inlineStr"/>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-WOYygWb2xY</t>
+        </is>
+      </c>
     </row>
     <row r="1245">
       <c r="A1245" t="inlineStr">
@@ -43191,7 +44271,11 @@
         </is>
       </c>
       <c r="G1247" t="inlineStr"/>
-      <c r="H1247" t="inlineStr"/>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bNBAFRTblGQ</t>
+        </is>
+      </c>
     </row>
     <row r="1248">
       <c r="A1248" t="inlineStr">
@@ -43225,7 +44309,11 @@
         </is>
       </c>
       <c r="G1248" t="inlineStr"/>
-      <c r="H1248" t="inlineStr"/>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bNBAFRTblGQ</t>
+        </is>
+      </c>
     </row>
     <row r="1249">
       <c r="A1249" t="inlineStr">
@@ -43327,7 +44415,11 @@
         </is>
       </c>
       <c r="G1251" t="inlineStr"/>
-      <c r="H1251" t="inlineStr"/>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9KeCW0jnXyQ</t>
+        </is>
+      </c>
     </row>
     <row r="1252">
       <c r="A1252" t="inlineStr">
@@ -43361,7 +44453,11 @@
         </is>
       </c>
       <c r="G1252" t="inlineStr"/>
-      <c r="H1252" t="inlineStr"/>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9KeCW0jnXyQ</t>
+        </is>
+      </c>
     </row>
     <row r="1253">
       <c r="A1253" t="inlineStr">
@@ -43395,7 +44491,11 @@
         </is>
       </c>
       <c r="G1253" t="inlineStr"/>
-      <c r="H1253" t="inlineStr"/>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9KeCW0jnXyQ</t>
+        </is>
+      </c>
     </row>
     <row r="1254">
       <c r="A1254" t="inlineStr">
@@ -43463,7 +44563,11 @@
         </is>
       </c>
       <c r="G1255" t="inlineStr"/>
-      <c r="H1255" t="inlineStr"/>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1256">
       <c r="A1256" t="inlineStr">
@@ -43497,7 +44601,11 @@
         </is>
       </c>
       <c r="G1256" t="inlineStr"/>
-      <c r="H1256" t="inlineStr"/>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1257">
       <c r="A1257" t="inlineStr">
@@ -43565,7 +44673,11 @@
         </is>
       </c>
       <c r="G1258" t="inlineStr"/>
-      <c r="H1258" t="inlineStr"/>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1259">
       <c r="A1259" t="inlineStr">
@@ -43599,7 +44711,11 @@
         </is>
       </c>
       <c r="G1259" t="inlineStr"/>
-      <c r="H1259" t="inlineStr"/>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1260">
       <c r="A1260" t="inlineStr">
@@ -43633,7 +44749,11 @@
         </is>
       </c>
       <c r="G1260" t="inlineStr"/>
-      <c r="H1260" t="inlineStr"/>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1261">
       <c r="A1261" t="inlineStr">
@@ -43667,7 +44787,11 @@
         </is>
       </c>
       <c r="G1261" t="inlineStr"/>
-      <c r="H1261" t="inlineStr"/>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WFLjkM7Agwk</t>
+        </is>
+      </c>
     </row>
     <row r="1262">
       <c r="A1262" t="inlineStr">
@@ -43701,7 +44825,11 @@
         </is>
       </c>
       <c r="G1262" t="inlineStr"/>
-      <c r="H1262" t="inlineStr"/>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WFLjkM7Agwk</t>
+        </is>
+      </c>
     </row>
     <row r="1263">
       <c r="A1263" t="inlineStr">
@@ -43735,7 +44863,11 @@
         </is>
       </c>
       <c r="G1263" t="inlineStr"/>
-      <c r="H1263" t="inlineStr"/>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IerotDC6VHg</t>
+        </is>
+      </c>
     </row>
     <row r="1264">
       <c r="A1264" t="inlineStr">
@@ -43769,7 +44901,11 @@
         </is>
       </c>
       <c r="G1264" t="inlineStr"/>
-      <c r="H1264" t="inlineStr"/>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IerotDC6VHg</t>
+        </is>
+      </c>
     </row>
     <row r="1265">
       <c r="A1265" t="inlineStr">
@@ -43803,7 +44939,11 @@
         </is>
       </c>
       <c r="G1265" t="inlineStr"/>
-      <c r="H1265" t="inlineStr"/>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OiBaQoOsbXU</t>
+        </is>
+      </c>
     </row>
     <row r="1266">
       <c r="A1266" t="inlineStr">
@@ -43837,7 +44977,11 @@
         </is>
       </c>
       <c r="G1266" t="inlineStr"/>
-      <c r="H1266" t="inlineStr"/>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fwaqdNrw_HQ</t>
+        </is>
+      </c>
     </row>
     <row r="1267">
       <c r="A1267" t="inlineStr">
@@ -43871,7 +45015,11 @@
         </is>
       </c>
       <c r="G1267" t="inlineStr"/>
-      <c r="H1267" t="inlineStr"/>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1268">
       <c r="A1268" t="inlineStr">
@@ -43905,7 +45053,11 @@
         </is>
       </c>
       <c r="G1268" t="inlineStr"/>
-      <c r="H1268" t="inlineStr"/>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1269">
       <c r="A1269" t="inlineStr">
@@ -43939,7 +45091,11 @@
         </is>
       </c>
       <c r="G1269" t="inlineStr"/>
-      <c r="H1269" t="inlineStr"/>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1270">
       <c r="A1270" t="inlineStr">
@@ -43973,7 +45129,11 @@
         </is>
       </c>
       <c r="G1270" t="inlineStr"/>
-      <c r="H1270" t="inlineStr"/>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1271">
       <c r="A1271" t="inlineStr">
@@ -44007,7 +45167,11 @@
         </is>
       </c>
       <c r="G1271" t="inlineStr"/>
-      <c r="H1271" t="inlineStr"/>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1272">
       <c r="A1272" t="inlineStr">
@@ -44041,7 +45205,11 @@
         </is>
       </c>
       <c r="G1272" t="inlineStr"/>
-      <c r="H1272" t="inlineStr"/>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1273">
       <c r="A1273" t="inlineStr">
@@ -44075,7 +45243,11 @@
         </is>
       </c>
       <c r="G1273" t="inlineStr"/>
-      <c r="H1273" t="inlineStr"/>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1274">
       <c r="A1274" t="inlineStr">
@@ -44109,7 +45281,11 @@
         </is>
       </c>
       <c r="G1274" t="inlineStr"/>
-      <c r="H1274" t="inlineStr"/>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1275">
       <c r="A1275" t="inlineStr">
@@ -44143,7 +45319,11 @@
         </is>
       </c>
       <c r="G1275" t="inlineStr"/>
-      <c r="H1275" t="inlineStr"/>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1276">
       <c r="A1276" t="inlineStr">
@@ -44177,7 +45357,11 @@
         </is>
       </c>
       <c r="G1276" t="inlineStr"/>
-      <c r="H1276" t="inlineStr"/>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1277">
       <c r="A1277" t="inlineStr">
@@ -44211,7 +45395,11 @@
         </is>
       </c>
       <c r="G1277" t="inlineStr"/>
-      <c r="H1277" t="inlineStr"/>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1278">
       <c r="A1278" t="inlineStr">
@@ -44245,7 +45433,11 @@
         </is>
       </c>
       <c r="G1278" t="inlineStr"/>
-      <c r="H1278" t="inlineStr"/>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1279">
       <c r="A1279" t="inlineStr">
@@ -44279,7 +45471,11 @@
         </is>
       </c>
       <c r="G1279" t="inlineStr"/>
-      <c r="H1279" t="inlineStr"/>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bW21J73kR_M</t>
+        </is>
+      </c>
     </row>
     <row r="1280">
       <c r="A1280" t="inlineStr">
@@ -44313,7 +45509,11 @@
         </is>
       </c>
       <c r="G1280" t="inlineStr"/>
-      <c r="H1280" t="inlineStr"/>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1281">
       <c r="A1281" t="inlineStr">
@@ -44347,7 +45547,11 @@
         </is>
       </c>
       <c r="G1281" t="inlineStr"/>
-      <c r="H1281" t="inlineStr"/>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1282">
       <c r="A1282" t="inlineStr">
@@ -44381,7 +45585,11 @@
         </is>
       </c>
       <c r="G1282" t="inlineStr"/>
-      <c r="H1282" t="inlineStr"/>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bxL3Dq06tW8</t>
+        </is>
+      </c>
     </row>
     <row r="1283">
       <c r="A1283" t="inlineStr">
@@ -44415,7 +45623,11 @@
         </is>
       </c>
       <c r="G1283" t="inlineStr"/>
-      <c r="H1283" t="inlineStr"/>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bxL3Dq06tW8</t>
+        </is>
+      </c>
     </row>
     <row r="1284">
       <c r="A1284" t="inlineStr">
@@ -44449,7 +45661,11 @@
         </is>
       </c>
       <c r="G1284" t="inlineStr"/>
-      <c r="H1284" t="inlineStr"/>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1285">
       <c r="A1285" t="inlineStr">
@@ -44483,7 +45699,11 @@
         </is>
       </c>
       <c r="G1285" t="inlineStr"/>
-      <c r="H1285" t="inlineStr"/>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f5s7O9b7M1g</t>
+        </is>
+      </c>
     </row>
     <row r="1286">
       <c r="A1286" t="inlineStr">
@@ -44517,7 +45737,11 @@
         </is>
       </c>
       <c r="G1286" t="inlineStr"/>
-      <c r="H1286" t="inlineStr"/>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=f5s7O9b7M1g</t>
+        </is>
+      </c>
     </row>
     <row r="1287">
       <c r="A1287" t="inlineStr">
@@ -44551,7 +45775,11 @@
         </is>
       </c>
       <c r="G1287" t="inlineStr"/>
-      <c r="H1287" t="inlineStr"/>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1288">
       <c r="A1288" t="inlineStr">
@@ -44585,7 +45813,11 @@
         </is>
       </c>
       <c r="G1288" t="inlineStr"/>
-      <c r="H1288" t="inlineStr"/>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1289">
       <c r="A1289" t="inlineStr">
@@ -44619,7 +45851,11 @@
         </is>
       </c>
       <c r="G1289" t="inlineStr"/>
-      <c r="H1289" t="inlineStr"/>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1290">
       <c r="A1290" t="inlineStr">
@@ -44653,7 +45889,11 @@
         </is>
       </c>
       <c r="G1290" t="inlineStr"/>
-      <c r="H1290" t="inlineStr"/>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1291">
       <c r="A1291" t="inlineStr">
@@ -44687,7 +45927,11 @@
         </is>
       </c>
       <c r="G1291" t="inlineStr"/>
-      <c r="H1291" t="inlineStr"/>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_FOjMSGFk_4</t>
+        </is>
+      </c>
     </row>
     <row r="1292">
       <c r="A1292" t="inlineStr">
@@ -44721,7 +45965,11 @@
         </is>
       </c>
       <c r="G1292" t="inlineStr"/>
-      <c r="H1292" t="inlineStr"/>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1293">
       <c r="A1293" t="inlineStr">
@@ -44755,7 +46003,11 @@
         </is>
       </c>
       <c r="G1293" t="inlineStr"/>
-      <c r="H1293" t="inlineStr"/>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1294">
       <c r="A1294" t="inlineStr">
@@ -44789,7 +46041,11 @@
         </is>
       </c>
       <c r="G1294" t="inlineStr"/>
-      <c r="H1294" t="inlineStr"/>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1295">
       <c r="A1295" t="inlineStr">
@@ -44823,7 +46079,11 @@
         </is>
       </c>
       <c r="G1295" t="inlineStr"/>
-      <c r="H1295" t="inlineStr"/>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SNGFWfNKC1s</t>
+        </is>
+      </c>
     </row>
     <row r="1296">
       <c r="A1296" t="inlineStr">
@@ -44857,7 +46117,11 @@
         </is>
       </c>
       <c r="G1296" t="inlineStr"/>
-      <c r="H1296" t="inlineStr"/>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-WOYygWb2xY</t>
+        </is>
+      </c>
     </row>
     <row r="1297">
       <c r="A1297" t="inlineStr">
@@ -44891,7 +46155,11 @@
         </is>
       </c>
       <c r="G1297" t="inlineStr"/>
-      <c r="H1297" t="inlineStr"/>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SZT0BYl2MIc</t>
+        </is>
+      </c>
     </row>
     <row r="1298">
       <c r="A1298" t="inlineStr">
@@ -44925,7 +46193,11 @@
         </is>
       </c>
       <c r="G1298" t="inlineStr"/>
-      <c r="H1298" t="inlineStr"/>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SZT0BYl2MIc</t>
+        </is>
+      </c>
     </row>
     <row r="1299">
       <c r="A1299" t="inlineStr">
@@ -44959,7 +46231,11 @@
         </is>
       </c>
       <c r="G1299" t="inlineStr"/>
-      <c r="H1299" t="inlineStr"/>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yVuzytn2kks</t>
+        </is>
+      </c>
     </row>
     <row r="1300">
       <c r="A1300" t="inlineStr">
@@ -44993,7 +46269,11 @@
         </is>
       </c>
       <c r="G1300" t="inlineStr"/>
-      <c r="H1300" t="inlineStr"/>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yVuzytn2kks</t>
+        </is>
+      </c>
     </row>
     <row r="1301">
       <c r="A1301" t="inlineStr">
@@ -45027,7 +46307,11 @@
         </is>
       </c>
       <c r="G1301" t="inlineStr"/>
-      <c r="H1301" t="inlineStr"/>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1302">
       <c r="A1302" t="inlineStr">
@@ -45061,7 +46345,11 @@
         </is>
       </c>
       <c r="G1302" t="inlineStr"/>
-      <c r="H1302" t="inlineStr"/>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1303">
       <c r="A1303" t="inlineStr">
@@ -45095,7 +46383,11 @@
         </is>
       </c>
       <c r="G1303" t="inlineStr"/>
-      <c r="H1303" t="inlineStr"/>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1304">
       <c r="A1304" t="inlineStr">
@@ -45129,7 +46421,11 @@
         </is>
       </c>
       <c r="G1304" t="inlineStr"/>
-      <c r="H1304" t="inlineStr"/>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1305">
       <c r="A1305" t="inlineStr">
@@ -45163,7 +46459,11 @@
         </is>
       </c>
       <c r="G1305" t="inlineStr"/>
-      <c r="H1305" t="inlineStr"/>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1306">
       <c r="A1306" t="inlineStr">
@@ -45201,7 +46501,11 @@
           <t>https://www.imex.cl/fichas/SWPTF02.pdf</t>
         </is>
       </c>
-      <c r="H1306" t="inlineStr"/>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1307">
       <c r="A1307" t="inlineStr">
@@ -45239,7 +46543,11 @@
           <t>https://www.imex.cl/fichas/SWPTM02.pdf</t>
         </is>
       </c>
-      <c r="H1307" t="inlineStr"/>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1308">
       <c r="A1308" t="inlineStr">
@@ -45273,7 +46581,11 @@
         </is>
       </c>
       <c r="G1308" t="inlineStr"/>
-      <c r="H1308" t="inlineStr"/>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1309">
       <c r="A1309" t="inlineStr">
@@ -45311,7 +46623,11 @@
           <t>https://www.imex.cl/fichas/SWPTF01.pdf</t>
         </is>
       </c>
-      <c r="H1309" t="inlineStr"/>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1310">
       <c r="A1310" t="inlineStr">
@@ -45349,7 +46665,11 @@
           <t>https://www.imex.cl/fichas/SWPTM01.pdf</t>
         </is>
       </c>
-      <c r="H1310" t="inlineStr"/>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1311">
       <c r="A1311" t="inlineStr">
@@ -45383,7 +46703,11 @@
         </is>
       </c>
       <c r="G1311" t="inlineStr"/>
-      <c r="H1311" t="inlineStr"/>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1312">
       <c r="A1312" t="inlineStr">
@@ -45421,7 +46745,11 @@
           <t>https://www.imex.cl/fichas/SWPTF05.pdf</t>
         </is>
       </c>
-      <c r="H1312" t="inlineStr"/>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1313">
       <c r="A1313" t="inlineStr">
@@ -45455,7 +46783,11 @@
         </is>
       </c>
       <c r="G1313" t="inlineStr"/>
-      <c r="H1313" t="inlineStr"/>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1314">
       <c r="A1314" t="inlineStr">
@@ -45489,7 +46821,11 @@
         </is>
       </c>
       <c r="G1314" t="inlineStr"/>
-      <c r="H1314" t="inlineStr"/>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1315">
       <c r="A1315" t="inlineStr">
@@ -45527,7 +46863,11 @@
           <t>https://www.imex.cl/fichas/SWPTM05.pdf</t>
         </is>
       </c>
-      <c r="H1315" t="inlineStr"/>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1316">
       <c r="A1316" t="inlineStr">
@@ -45561,7 +46901,11 @@
         </is>
       </c>
       <c r="G1316" t="inlineStr"/>
-      <c r="H1316" t="inlineStr"/>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1317">
       <c r="A1317" t="inlineStr">
@@ -45595,7 +46939,11 @@
         </is>
       </c>
       <c r="G1317" t="inlineStr"/>
-      <c r="H1317" t="inlineStr"/>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fsck-m92OZk</t>
+        </is>
+      </c>
     </row>
     <row r="1318">
       <c r="A1318" t="inlineStr">
@@ -45629,7 +46977,11 @@
         </is>
       </c>
       <c r="G1318" t="inlineStr"/>
-      <c r="H1318" t="inlineStr"/>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1319">
       <c r="A1319" t="inlineStr">
@@ -45663,7 +47015,11 @@
         </is>
       </c>
       <c r="G1319" t="inlineStr"/>
-      <c r="H1319" t="inlineStr"/>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1320">
       <c r="A1320" t="inlineStr">
@@ -45697,7 +47053,11 @@
         </is>
       </c>
       <c r="G1320" t="inlineStr"/>
-      <c r="H1320" t="inlineStr"/>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1321">
       <c r="A1321" t="inlineStr">
@@ -45731,7 +47091,11 @@
         </is>
       </c>
       <c r="G1321" t="inlineStr"/>
-      <c r="H1321" t="inlineStr"/>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1322">
       <c r="A1322" t="inlineStr">
@@ -45769,7 +47133,11 @@
           <t>https://www.imex.cl/fichas/SWPTF03.pdf</t>
         </is>
       </c>
-      <c r="H1322" t="inlineStr"/>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1323">
       <c r="A1323" t="inlineStr">
@@ -45807,7 +47175,11 @@
           <t>https://www.imex.cl/fichas/SWPTM03.pdf</t>
         </is>
       </c>
-      <c r="H1323" t="inlineStr"/>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1324">
       <c r="A1324" t="inlineStr">
@@ -45841,7 +47213,11 @@
         </is>
       </c>
       <c r="G1324" t="inlineStr"/>
-      <c r="H1324" t="inlineStr"/>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1325">
       <c r="A1325" t="inlineStr">
@@ -45875,7 +47251,11 @@
         </is>
       </c>
       <c r="G1325" t="inlineStr"/>
-      <c r="H1325" t="inlineStr"/>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1326">
       <c r="A1326" t="inlineStr">
@@ -45909,7 +47289,11 @@
         </is>
       </c>
       <c r="G1326" t="inlineStr"/>
-      <c r="H1326" t="inlineStr"/>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1327">
       <c r="A1327" t="inlineStr">
@@ -45943,7 +47327,11 @@
         </is>
       </c>
       <c r="G1327" t="inlineStr"/>
-      <c r="H1327" t="inlineStr"/>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1328">
       <c r="A1328" t="inlineStr">
@@ -45981,7 +47369,11 @@
           <t>https://www.imex.cl/fichas/SWPTF04.pdf</t>
         </is>
       </c>
-      <c r="H1328" t="inlineStr"/>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1329">
       <c r="A1329" t="inlineStr">
@@ -46019,7 +47411,11 @@
           <t>https://www.imex.cl/fichas/SWPTM04.pdf</t>
         </is>
       </c>
-      <c r="H1329" t="inlineStr"/>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zORE-l7HIdo</t>
+        </is>
+      </c>
     </row>
     <row r="1330">
       <c r="A1330" t="inlineStr">
@@ -46053,7 +47449,11 @@
         </is>
       </c>
       <c r="G1330" t="inlineStr"/>
-      <c r="H1330" t="inlineStr"/>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bHPUThy-GGc</t>
+        </is>
+      </c>
     </row>
     <row r="1331">
       <c r="A1331" t="inlineStr">
@@ -46087,7 +47487,11 @@
         </is>
       </c>
       <c r="G1331" t="inlineStr"/>
-      <c r="H1331" t="inlineStr"/>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1332">
       <c r="A1332" t="inlineStr">
@@ -46121,7 +47525,11 @@
         </is>
       </c>
       <c r="G1332" t="inlineStr"/>
-      <c r="H1332" t="inlineStr"/>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1333">
       <c r="A1333" t="inlineStr">
@@ -46155,7 +47563,11 @@
         </is>
       </c>
       <c r="G1333" t="inlineStr"/>
-      <c r="H1333" t="inlineStr"/>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1334">
       <c r="A1334" t="inlineStr">
@@ -46189,7 +47601,11 @@
         </is>
       </c>
       <c r="G1334" t="inlineStr"/>
-      <c r="H1334" t="inlineStr"/>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1335">
       <c r="A1335" t="inlineStr">
@@ -46223,7 +47639,11 @@
         </is>
       </c>
       <c r="G1335" t="inlineStr"/>
-      <c r="H1335" t="inlineStr"/>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-cgx7mhxof4</t>
+        </is>
+      </c>
     </row>
     <row r="1336">
       <c r="A1336" t="inlineStr">
@@ -46257,7 +47677,11 @@
         </is>
       </c>
       <c r="G1336" t="inlineStr"/>
-      <c r="H1336" t="inlineStr"/>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HMVEP73WGLs</t>
+        </is>
+      </c>
     </row>
     <row r="1337">
       <c r="A1337" t="inlineStr">
@@ -46291,7 +47715,11 @@
         </is>
       </c>
       <c r="G1337" t="inlineStr"/>
-      <c r="H1337" t="inlineStr"/>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HMVEP73WGLs</t>
+        </is>
+      </c>
     </row>
     <row r="1338">
       <c r="A1338" t="inlineStr">
@@ -46325,7 +47753,11 @@
         </is>
       </c>
       <c r="G1338" t="inlineStr"/>
-      <c r="H1338" t="inlineStr"/>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HMVEP73WGLs</t>
+        </is>
+      </c>
     </row>
     <row r="1339">
       <c r="A1339" t="inlineStr">
@@ -46359,7 +47791,11 @@
         </is>
       </c>
       <c r="G1339" t="inlineStr"/>
-      <c r="H1339" t="inlineStr"/>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HMVEP73WGLs</t>
+        </is>
+      </c>
     </row>
     <row r="1340">
       <c r="A1340" t="inlineStr">
@@ -46393,7 +47829,11 @@
         </is>
       </c>
       <c r="G1340" t="inlineStr"/>
-      <c r="H1340" t="inlineStr"/>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HMVEP73WGLs</t>
+        </is>
+      </c>
     </row>
     <row r="1341">
       <c r="A1341" t="inlineStr">

</xml_diff>